<commit_message>
Normaliza aliases de jogadores
</commit_message>
<xml_diff>
--- a/2x2 presencial.xlsx
+++ b/2x2 presencial.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Edd\Desktop\Codes\Liga preconauta\preconauta-league\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E699EA91-E3A6-49B4-A562-386900E5994F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53AECC94-D0D6-4433-8E56-93E566876930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="298">
   <si>
     <t>evento</t>
   </si>
@@ -645,9 +645,6 @@
     <t>Sônia</t>
   </si>
   <si>
-    <t>Guff</t>
-  </si>
-  <si>
     <t>Chaca &amp; Susan</t>
   </si>
   <si>
@@ -771,12 +768,6 @@
     <t>Maelstrom Arcano</t>
   </si>
   <si>
-    <t>Pirmari Artistry</t>
-  </si>
-  <si>
-    <t>Velociramptor</t>
-  </si>
-  <si>
     <t>Zangalli &amp; Chueiry</t>
   </si>
   <si>
@@ -889,9 +880,6 @@
   </si>
   <si>
     <t>Denilson</t>
-  </si>
-  <si>
-    <t>Pantlaza</t>
   </si>
   <si>
     <t>Oscar &amp; Vinicius</t>
@@ -4095,7 +4083,7 @@
         <v>191</v>
       </c>
       <c r="F130" t="s">
-        <v>201</v>
+        <v>254</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
@@ -4103,19 +4091,19 @@
         <v>193</v>
       </c>
       <c r="B131" t="s">
+        <v>201</v>
+      </c>
+      <c r="C131" t="s">
         <v>202</v>
       </c>
-      <c r="C131" t="s">
+      <c r="D131" t="s">
         <v>203</v>
-      </c>
-      <c r="D131" t="s">
-        <v>204</v>
       </c>
       <c r="E131" t="s">
         <v>19</v>
       </c>
       <c r="F131" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
@@ -4123,16 +4111,16 @@
         <v>193</v>
       </c>
       <c r="B132" t="s">
+        <v>205</v>
+      </c>
+      <c r="C132" t="s">
         <v>206</v>
       </c>
-      <c r="C132" t="s">
+      <c r="D132" t="s">
         <v>207</v>
       </c>
-      <c r="D132" t="s">
+      <c r="E132" t="s">
         <v>208</v>
-      </c>
-      <c r="E132" t="s">
-        <v>209</v>
       </c>
       <c r="F132" t="s">
         <v>106</v>
@@ -4143,19 +4131,19 @@
         <v>193</v>
       </c>
       <c r="B133" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C133" t="s">
         <v>194</v>
       </c>
       <c r="D133" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E133" t="s">
         <v>129</v>
       </c>
       <c r="F133" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
@@ -4163,13 +4151,13 @@
         <v>193</v>
       </c>
       <c r="B134" t="s">
+        <v>212</v>
+      </c>
+      <c r="C134" t="s">
         <v>213</v>
       </c>
-      <c r="C134" t="s">
+      <c r="D134" t="s">
         <v>214</v>
-      </c>
-      <c r="D134" t="s">
-        <v>215</v>
       </c>
       <c r="E134" t="s">
         <v>29</v>
@@ -4183,13 +4171,13 @@
         <v>193</v>
       </c>
       <c r="B135" t="s">
+        <v>215</v>
+      </c>
+      <c r="C135" t="s">
         <v>216</v>
       </c>
-      <c r="C135" t="s">
+      <c r="D135" t="s">
         <v>217</v>
-      </c>
-      <c r="D135" t="s">
-        <v>218</v>
       </c>
       <c r="E135" t="s">
         <v>148</v>
@@ -4203,24 +4191,24 @@
         <v>193</v>
       </c>
       <c r="B136" t="s">
+        <v>218</v>
+      </c>
+      <c r="C136" t="s">
         <v>219</v>
       </c>
-      <c r="C136" t="s">
+      <c r="D136" t="s">
         <v>220</v>
-      </c>
-      <c r="D136" t="s">
-        <v>221</v>
       </c>
       <c r="E136" t="s">
         <v>162</v>
       </c>
       <c r="F136" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B137" t="s">
         <v>38</v>
@@ -4240,7 +4228,7 @@
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B138" t="s">
         <v>25</v>
@@ -4249,7 +4237,7 @@
         <v>160</v>
       </c>
       <c r="D138" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E138" t="s">
         <v>59</v>
@@ -4260,7 +4248,7 @@
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B139" t="s">
         <v>94</v>
@@ -4280,7 +4268,7 @@
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B140" t="s">
         <v>112</v>
@@ -4300,7 +4288,7 @@
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B141" t="s">
         <v>103</v>
@@ -4309,10 +4297,10 @@
         <v>169</v>
       </c>
       <c r="D141" t="s">
+        <v>224</v>
+      </c>
+      <c r="E141" t="s">
         <v>225</v>
-      </c>
-      <c r="E141" t="s">
-        <v>226</v>
       </c>
       <c r="F141" t="s">
         <v>150</v>
@@ -4320,13 +4308,13 @@
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B142" t="s">
+        <v>226</v>
+      </c>
+      <c r="C142" t="s">
         <v>227</v>
-      </c>
-      <c r="C142" t="s">
-        <v>228</v>
       </c>
       <c r="D142" t="s">
         <v>197</v>
@@ -4340,16 +4328,16 @@
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B143" t="s">
         <v>53</v>
       </c>
       <c r="C143" t="s">
+        <v>228</v>
+      </c>
+      <c r="D143" t="s">
         <v>229</v>
-      </c>
-      <c r="D143" t="s">
-        <v>230</v>
       </c>
       <c r="E143" t="s">
         <v>48</v>
@@ -4360,10 +4348,10 @@
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B144" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C144" t="s">
         <v>173</v>
@@ -4380,7 +4368,7 @@
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B145" t="s">
         <v>189</v>
@@ -4400,16 +4388,16 @@
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B146" t="s">
+        <v>201</v>
+      </c>
+      <c r="C146" t="s">
         <v>202</v>
       </c>
-      <c r="C146" t="s">
+      <c r="D146" t="s">
         <v>203</v>
-      </c>
-      <c r="D146" t="s">
-        <v>204</v>
       </c>
       <c r="E146" t="s">
         <v>19</v>
@@ -4420,16 +4408,16 @@
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B147" t="s">
+        <v>205</v>
+      </c>
+      <c r="C147" t="s">
         <v>206</v>
       </c>
-      <c r="C147" t="s">
+      <c r="D147" t="s">
         <v>207</v>
-      </c>
-      <c r="D147" t="s">
-        <v>208</v>
       </c>
       <c r="E147" t="s">
         <v>106</v>
@@ -4440,16 +4428,16 @@
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B148" t="s">
+        <v>232</v>
+      </c>
+      <c r="C148" t="s">
         <v>233</v>
       </c>
-      <c r="C148" t="s">
+      <c r="D148" t="s">
         <v>234</v>
-      </c>
-      <c r="D148" t="s">
-        <v>235</v>
       </c>
       <c r="E148" t="s">
         <v>27</v>
@@ -4460,16 +4448,16 @@
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B149" t="s">
         <v>84</v>
       </c>
       <c r="C149" t="s">
+        <v>235</v>
+      </c>
+      <c r="D149" t="s">
         <v>236</v>
-      </c>
-      <c r="D149" t="s">
-        <v>237</v>
       </c>
       <c r="E149" t="s">
         <v>17</v>
@@ -4480,7 +4468,7 @@
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B150" t="s">
         <v>38</v>
@@ -4500,7 +4488,7 @@
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B151" t="s">
         <v>25</v>
@@ -4509,7 +4497,7 @@
         <v>160</v>
       </c>
       <c r="D151" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E151" t="s">
         <v>15</v>
@@ -4520,7 +4508,7 @@
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B152" t="s">
         <v>103</v>
@@ -4529,18 +4517,18 @@
         <v>169</v>
       </c>
       <c r="D152" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E152" t="s">
+        <v>240</v>
+      </c>
+      <c r="F152" t="s">
         <v>241</v>
-      </c>
-      <c r="F152" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B153" t="s">
         <v>98</v>
@@ -4552,15 +4540,15 @@
         <v>167</v>
       </c>
       <c r="E153" t="s">
-        <v>243</v>
+        <v>108</v>
       </c>
       <c r="F153" t="s">
-        <v>244</v>
+        <v>17</v>
       </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B154" t="s">
         <v>94</v>
@@ -4580,36 +4568,36 @@
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B155" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="C155" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D155" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E155" t="s">
         <v>31</v>
       </c>
       <c r="F155" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B156" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="C156" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D156" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E156" t="s">
         <v>149</v>
@@ -4620,16 +4608,16 @@
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B157" t="s">
+        <v>201</v>
+      </c>
+      <c r="C157" t="s">
         <v>202</v>
       </c>
-      <c r="C157" t="s">
+      <c r="D157" t="s">
         <v>203</v>
-      </c>
-      <c r="D157" t="s">
-        <v>204</v>
       </c>
       <c r="E157" t="s">
         <v>19</v>
@@ -4640,7 +4628,7 @@
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B158" t="s">
         <v>189</v>
@@ -4660,13 +4648,13 @@
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B159" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C159" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D159" t="s">
         <v>161</v>
@@ -4680,16 +4668,16 @@
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B160" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="C160" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="D160" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="E160" t="s">
         <v>39</v>
@@ -4700,16 +4688,16 @@
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B161" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="C161" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D161" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E161" t="s">
         <v>31</v>
@@ -4720,7 +4708,7 @@
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B162" t="s">
         <v>143</v>
@@ -4740,27 +4728,27 @@
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B163" t="s">
         <v>53</v>
       </c>
       <c r="C163" t="s">
+        <v>228</v>
+      </c>
+      <c r="D163" t="s">
         <v>229</v>
-      </c>
-      <c r="D163" t="s">
-        <v>230</v>
       </c>
       <c r="E163" t="s">
         <v>39</v>
       </c>
       <c r="F163" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B164" t="s">
         <v>103</v>
@@ -4769,7 +4757,7 @@
         <v>169</v>
       </c>
       <c r="D164" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E164" t="s">
         <v>150</v>
@@ -4780,7 +4768,7 @@
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B165" t="s">
         <v>111</v>
@@ -4800,7 +4788,7 @@
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B166" t="s">
         <v>38</v>
@@ -4820,19 +4808,19 @@
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B167" t="s">
+        <v>201</v>
+      </c>
+      <c r="C167" t="s">
         <v>202</v>
       </c>
-      <c r="C167" t="s">
+      <c r="D167" t="s">
         <v>203</v>
       </c>
-      <c r="D167" t="s">
-        <v>204</v>
-      </c>
       <c r="E167" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="F167" t="s">
         <v>149</v>
@@ -4840,16 +4828,16 @@
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B168" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C168" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D168" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="E168" t="s">
         <v>17</v>
@@ -4860,27 +4848,27 @@
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B169" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C169" t="s">
         <v>187</v>
       </c>
       <c r="D169" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E169" t="s">
         <v>15</v>
       </c>
       <c r="F169" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B170" t="s">
         <v>112</v>
@@ -4900,16 +4888,16 @@
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B171" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C171" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="D171" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="E171" t="s">
         <v>49</v>
@@ -4920,19 +4908,19 @@
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B172" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="C172" t="s">
         <v>194</v>
       </c>
       <c r="D172" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E172" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="F172" t="s">
         <v>149</v>
@@ -4940,7 +4928,7 @@
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B173" t="s">
         <v>38</v>
@@ -4960,16 +4948,16 @@
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B174" t="s">
         <v>146</v>
       </c>
       <c r="C174" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D174" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="E174" t="s">
         <v>149</v>
@@ -4980,19 +4968,19 @@
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B175" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="C175" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D175" t="s">
         <v>170</v>
       </c>
       <c r="E175" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="F175" t="s">
         <v>15</v>
@@ -5000,7 +4988,7 @@
     </row>
     <row r="176" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B176" t="s">
         <v>143</v>
@@ -5015,24 +5003,24 @@
         <v>130</v>
       </c>
       <c r="F176" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B177" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="C177" t="s">
         <v>168</v>
       </c>
       <c r="D177" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="E177" t="s">
-        <v>283</v>
+        <v>17</v>
       </c>
       <c r="F177" t="s">
         <v>108</v>
@@ -5040,16 +5028,16 @@
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B178" t="s">
+        <v>201</v>
+      </c>
+      <c r="C178" t="s">
         <v>202</v>
       </c>
-      <c r="C178" t="s">
+      <c r="D178" t="s">
         <v>203</v>
-      </c>
-      <c r="D178" t="s">
-        <v>204</v>
       </c>
       <c r="E178" t="s">
         <v>126</v>
@@ -5060,19 +5048,19 @@
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B179" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C179" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D179" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="E179" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F179" t="s">
         <v>27</v>
@@ -5080,7 +5068,7 @@
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B180" t="s">
         <v>189</v>
@@ -5100,16 +5088,16 @@
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B181" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="C181" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D181" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="E181" t="s">
         <v>162</v>
@@ -5120,19 +5108,19 @@
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B182" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="C182" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D182" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="E182" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="F182" t="s">
         <v>178</v>
@@ -5140,7 +5128,7 @@
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B183" s="1" t="s">
         <v>38</v>
@@ -5160,19 +5148,19 @@
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B184" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C184" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D184" s="1" t="s">
         <v>160</v>
       </c>
       <c r="E184" s="1" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="F184" t="s">
         <v>48</v>
@@ -5180,16 +5168,16 @@
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B185" s="1" t="s">
         <v>84</v>
       </c>
       <c r="C185" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="D185" s="1" t="s">
         <v>236</v>
-      </c>
-      <c r="D185" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="E185" t="s">
         <v>15</v>
@@ -5200,10 +5188,10 @@
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B186" s="1" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="C186" s="1" t="s">
         <v>187</v>
@@ -5215,21 +5203,21 @@
         <v>87</v>
       </c>
       <c r="F186" s="1" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B187" s="1" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C187" s="1" t="s">
         <v>194</v>
       </c>
       <c r="D187" s="1" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E187" s="1" t="s">
         <v>149</v>
@@ -5240,16 +5228,16 @@
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B188" s="1" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="C188" s="1" t="s">
         <v>168</v>
       </c>
       <c r="D188" s="1" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="E188" s="1" t="s">
         <v>17</v>
@@ -5260,16 +5248,16 @@
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B189" s="1" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="C189" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D189" s="1" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="E189" s="1" t="s">
         <v>163</v>
@@ -5280,13 +5268,13 @@
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B190" s="1" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="C190" s="1" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="D190" s="1" t="s">
         <v>165</v>
@@ -5300,13 +5288,13 @@
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B191" s="1" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="C191" s="1" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="D191" s="1" t="s">
         <v>179</v>
@@ -5362,19 +5350,19 @@
         <v>56</v>
       </c>
       <c r="B2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="C2" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E2" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="F2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -5405,16 +5393,16 @@
         <v>53</v>
       </c>
       <c r="C4" t="s">
+        <v>228</v>
+      </c>
+      <c r="D4" t="s">
         <v>229</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>253</v>
+      </c>
+      <c r="F4" t="s">
         <v>230</v>
-      </c>
-      <c r="E4" t="s">
-        <v>256</v>
-      </c>
-      <c r="F4" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -5428,13 +5416,13 @@
         <v>169</v>
       </c>
       <c r="D5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E5" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="F5" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -5482,16 +5470,16 @@
         <v>56</v>
       </c>
       <c r="B8" t="s">
+        <v>201</v>
+      </c>
+      <c r="C8" t="s">
         <v>202</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>203</v>
       </c>
-      <c r="D8" t="s">
-        <v>204</v>
-      </c>
       <c r="E8" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="F8" t="s">
         <v>149</v>
@@ -5502,19 +5490,19 @@
         <v>56</v>
       </c>
       <c r="B9" t="s">
+        <v>260</v>
+      </c>
+      <c r="C9" t="s">
+        <v>261</v>
+      </c>
+      <c r="D9" t="s">
+        <v>262</v>
+      </c>
+      <c r="E9" t="s">
+        <v>223</v>
+      </c>
+      <c r="F9" t="s">
         <v>263</v>
-      </c>
-      <c r="C9" t="s">
-        <v>264</v>
-      </c>
-      <c r="D9" t="s">
-        <v>265</v>
-      </c>
-      <c r="E9" t="s">
-        <v>224</v>
-      </c>
-      <c r="F9" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -5522,19 +5510,19 @@
         <v>56</v>
       </c>
       <c r="B10" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C10" t="s">
         <v>187</v>
       </c>
       <c r="D10" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E10" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="F10" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -5551,10 +5539,10 @@
         <v>168</v>
       </c>
       <c r="E11" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="F11" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -5562,19 +5550,19 @@
         <v>56</v>
       </c>
       <c r="B12" t="s">
+        <v>267</v>
+      </c>
+      <c r="C12" t="s">
+        <v>268</v>
+      </c>
+      <c r="D12" t="s">
+        <v>269</v>
+      </c>
+      <c r="E12" t="s">
         <v>270</v>
       </c>
-      <c r="C12" t="s">
+      <c r="F12" t="s">
         <v>271</v>
-      </c>
-      <c r="D12" t="s">
-        <v>272</v>
-      </c>
-      <c r="E12" t="s">
-        <v>273</v>
-      </c>
-      <c r="F12" t="s">
-        <v>274</v>
       </c>
     </row>
   </sheetData>

</xml_diff>